<commit_message>
sync: envy · 2026-08-11 14:54:00
</commit_message>
<xml_diff>
--- a/fase_1/salida/tabla_price.xlsx
+++ b/fase_1/salida/tabla_price.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="PS" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="PS" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -223,17 +223,193 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1f497d"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="eeece1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4f81bd"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="c0504d"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9bbb59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064a2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4bacc6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="f79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ff"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11.85"/>

</xml_diff>